<commit_message>
Progression BACHINGE24 v1.6 : planning à 5 séances
La séance du 14/10 après-midi est supprimée et ses cours passent dans la
séance 2. La séance 3 devient l'intégration sur le serveur. Mise à jour de
materiel_ISTP.md, BACHTECH24.md et CLAUDE.md, ajout du planning xlsx modifié,
de l'ancien planning et de la documentation Niryo Ned2.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/progression_pedagogique/seances_BACHINGE24.xlsx
+++ b/progression_pedagogique/seances_BACHINGE24.xlsx
@@ -20,32 +20,35 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
+  <si>
+    <t xml:space="preserve">Cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Groupe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Début</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matériel nécessaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">programme</t>
+  </si>
   <si>
     <t xml:space="preserve">Infrastructure client / serveur dans un contexte industriel</t>
   </si>
   <si>
-    <t xml:space="preserve">Groupe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Début</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">salle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matériel nécessaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">programme</t>
-  </si>
-  <si>
     <t xml:space="preserve">G1</t>
   </si>
   <si>
@@ -88,13 +91,13 @@
     <t xml:space="preserve">C1,07</t>
   </si>
   <si>
-    <t xml:space="preserve">Analyse, réalisation dossier et présentation, définition des tests de recette</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/10/2026 13:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/10/2026 17:00</t>
+    <t xml:space="preserve">Analyse, réalisation dossier et présentation, définition des tests de recette, Cours : protocole MQTT, rappel SQL, collecter les données du process dans base SQLite, Python, réaliser un site web et réaliser une API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/11/2026 08:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/11/2026 12:00</t>
   </si>
   <si>
     <t xml:space="preserve">D3,10</t>
@@ -103,16 +106,7 @@
     <t xml:space="preserve">serveur</t>
   </si>
   <si>
-    <t xml:space="preserve">Cours : protocole MQTT, rappel SQL, collecter les données du process dans base SQLite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09/11/2026 08:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09/11/2026 12:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cours : Python, réaliser un site web et réaliser une API</t>
+    <t xml:space="preserve">integration sur serveur</t>
   </si>
   <si>
     <t xml:space="preserve">17/11/2026 08:30</t>
@@ -131,6 +125,9 @@
   </si>
   <si>
     <t xml:space="preserve">17/11/2026 17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test_Infrastructure client / serveur dans un contexte industriel</t>
   </si>
   <si>
     <t xml:space="preserve">19/11/2026 13:30</t>
@@ -158,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -181,15 +178,10 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -240,36 +232,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -396,253 +380,248 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0"/>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>7</v>
+      <c r="A2" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="H3" s="5" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>16</v>
+      <c r="A4" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E4" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>27</v>
+      <c r="G6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>28</v>
+      <c r="A7" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>30</v>
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="0" t="s">
+      <c r="A8" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>34</v>
+      <c r="H8" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="0" t="s">
+      <c r="A9" s="0" t="s">
         <v>35</v>
       </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="C9" s="0" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="F9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>